<commit_message>
Remove place-name label from Excel sheets
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/offline-site/templates/points-workbook-template.xlsx
+++ b/offline-site/templates/points-workbook-template.xlsx
@@ -13,51 +13,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
-  <si>
-    <t>Название места</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+  <si>
+    <t>ФИО</t>
+  </si>
+  <si>
+    <t>Звание / должность</t>
+  </si>
+  <si>
+    <t>demo-point-001</t>
+  </si>
+  <si>
+    <t>Иванов Иван Иванович</t>
+  </si>
+  <si>
+    <t>Капитан</t>
+  </si>
+  <si>
+    <t>Петров Пётр Сергеевич</t>
+  </si>
+  <si>
+    <t>Инспектор</t>
+  </si>
+  <si>
+    <t>demo-point-002</t>
+  </si>
+  <si>
+    <t>Соколова Анна Викторовна</t>
+  </si>
+  <si>
+    <t>Кладовщик</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Лист</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
   <si>
     <t>КПП №1</t>
   </si>
   <si>
-    <t>demo-point-001</t>
-  </si>
-  <si>
-    <t>Иванов Иван Иванович</t>
-  </si>
-  <si>
-    <t>Капитан</t>
-  </si>
-  <si>
-    <t>Петров Пётр Сергеевич</t>
-  </si>
-  <si>
-    <t>Инспектор</t>
-  </si>
-  <si>
     <t>Склад №2</t>
-  </si>
-  <si>
-    <t>demo-point-002</t>
-  </si>
-  <si>
-    <t>Соколова Анна Викторовна</t>
-  </si>
-  <si>
-    <t>Кладовщик</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Лист</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -512,18 +515,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z1" t="s">
         <v>7</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -544,16 +547,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -561,7 +564,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C2">
         <v>420</v>
@@ -572,10 +575,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>1160</v>

</xml_diff>

<commit_message>
Keep place names without Excel label
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/offline-site/templates/points-workbook-template.xlsx
+++ b/offline-site/templates/points-workbook-template.xlsx
@@ -13,12 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
-  <si>
-    <t>ФИО</t>
-  </si>
-  <si>
-    <t>Звание / должность</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+  <si>
+    <t>КПП №1</t>
   </si>
   <si>
     <t>demo-point-001</t>
@@ -36,6 +33,9 @@
     <t>Инспектор</t>
   </si>
   <si>
+    <t>Склад №2</t>
+  </si>
+  <si>
     <t>demo-point-002</t>
   </si>
   <si>
@@ -55,12 +55,6 @@
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>КПП №1</t>
-  </si>
-  <si>
-    <t>Склад №2</t>
   </si>
 </sst>
 </file>
@@ -468,30 +462,28 @@
   </cols>
   <sheetData>
     <row r="1" ht="23" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>1</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -511,11 +503,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="23" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Z1" t="s">
         <v>7</v>
@@ -561,10 +551,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C2">
         <v>420</v>
@@ -578,7 +568,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>1160</v>

</xml_diff>

<commit_message>
Expand and optimize offline Eastern Europe map
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/offline-site/templates/points-workbook-template.xlsx
+++ b/offline-site/templates/points-workbook-template.xlsx
@@ -488,7 +488,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -521,21 +521,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="6" max="6" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
@@ -547,6 +548,9 @@
       </c>
       <c r="D1" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="F1" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -557,10 +561,10 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>420</v>
+        <v>512</v>
       </c>
       <c r="D2">
-        <v>580</v>
+        <v>658</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -571,14 +575,14 @@
         <v>6</v>
       </c>
       <c r="C3">
-        <v>1160</v>
+        <v>954</v>
       </c>
       <c r="D3">
-        <v>310</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>